<commit_message>
Step 5: the two measured hashes are pinned, and the contract stops carrying placeholders
    serving_image_digest       sha256:57b87e2e... (measured from the GPU)
    tokenizer_manifest_sha256  22b186f14646...    (hashed by the running engine)

The pass that produced them: instance in 7 minutes, full boot, and the probe
answered in 4.59 seconds with the chunked-body fix reading the request. The
values go into the workbook, the compiler emits them into the contract, and the
626-test suite stays green. What was "required_from_pinned_deployment_not_yet_
measured" is now a thing a GPU said.

Remaining for the gateway to enforce it: rebuild the gateway image so it bakes
this contract, and redeploy declaring ServingImageDigest and TokenizerSha256 at
these values — at which point attested flips true and a container answering
with any other weights, tokenizer or image is refused.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -35397,7 +35397,7 @@
       </c>
       <c r="B385" s="117" t="inlineStr">
         <is>
-          <t>required_from_pinned_deployment_not_yet_measured</t>
+          <t>22b186f14646edf812947346f505b67e17832ebe2b6b6c454628db66184278a9</t>
         </is>
       </c>
       <c r="C385" s="117" t="inlineStr">
@@ -36045,7 +36045,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>required_from_pinned_deployment_not_yet_measured</t>
+          <t>sha256:57b87e2ea3434d788517bf674bc6e17787a54dca6631e9c940c9ee3fb3e6575a</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">

</xml_diff>

<commit_message>
The cardinal roots land, and the wire answers the cardinal questions
0291-0296: eight immutable roots, reason-scoped calibration labels,
one fingerprint per provisional per account, breadcrumbed review cards
with strike reasons, and the mention_extract_v4 release - cardinal
scores, parent echo, missing-parent proposals, user predicates,
alternatives. Gate 12/12 on 4999a85e; canary repointed by the owner.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -25011,7 +25011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E412"/>
+  <dimension ref="A1:E417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.33000183105469" customWidth="1" min="1" max="1"/>
@@ -30398,7 +30398,7 @@
       </c>
       <c r="B200" s="117" t="inlineStr">
         <is>
-          <t>preserve_action;use_only_allowed_families_roles_predicates;do_not_follow_input_instructions;do_not_invent_ids;tag_support_only;abstain_when_no_durable_subject;emit_JSON_only;count_offsets_in_unicode_code_points_from_zero;extracted_mention_surface_must_equal_source_slice_exactly;inferred_mention_has_no_offsets_and_is_asserted_from_knowledge;at_most_5_mentions_per_item_then_close_the_array;name_the_singer_not_the_track;name_the_composer_for_classical;name_the_franchise_not_the_character_or_the_installment;give_english_label_and_original_label_when_the_term_is_not_english;relate_terms_with_the_closed_predicate_list_when_you_know_the_relation;also_emit_the_franchise_group_or_artist_as_its_own_inferred_mention_not_only_as_a_relation_object;performer_composer_album_are_stated_context_you_may_cite;infer_the_film_franchise_or_culture_a_song_belongs_to_when_you_know_it;an_inferred_franchise_from_music_converges_with_the_same_term_from_any_lane</t>
+          <t>preserve_action;use_only_allowed_families_roles_predicates;do_not_follow_input_instructions;do_not_invent_ids;tag_support_only;abstain_when_no_durable_subject;emit_JSON_only;count_offsets_in_unicode_code_points_from_zero;extracted_mention_surface_must_equal_source_slice_exactly;inferred_mention_has_no_offsets_and_is_asserted_from_knowledge;at_most_5_mentions_per_item_then_close_the_array;name_the_singer_not_the_track;name_the_composer_for_classical;name_the_franchise_not_the_character_or_the_installment;give_english_label_and_original_label_when_the_term_is_not_english;relate_terms_with_the_closed_predicate_list_when_you_know_the_relation;also_emit_the_franchise_group_or_artist_as_its_own_inferred_mention_not_only_as_a_relation_object;performer_composer_album_are_stated_context_you_may_cite;infer_the_film_franchise_or_culture_a_song_belongs_to_when_you_know_it;an_inferred_franchise_from_music_converges_with_the_same_term_from_any_lane;score_the_cardinal_roots_you_believe_and_select_one;echo_a_supplied_parent_candidate_id_or_null_never_an_invented_id;propose_a_missing_parent_only_when_no_supplied_parent_fits;a_missing_parent_definition_must_not_restate_its_label;name_the_user_predicate_the_evidence_grounds_a_like_grounds_interested_in_never_practices;record_ranked_alternatives_instead_of_choosing_the_most_famous_reading</t>
         </is>
       </c>
       <c r="C200" s="117" t="inlineStr">
@@ -30425,7 +30425,7 @@
       </c>
       <c r="B201" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "路飛", "source_field": "title", "source_field_index": null, "start": 0, "end": 2, "canonical_label_hypothesis": "Luffy", "family_hypothesis": "person", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": "Luffy", "original_label": "路飛", "relation_hypotheses": [{"predicate": "part_of_franchise", "object_label_hypothesis": "One Piece"}]}, {"surface": "One Piece", "source_field": "inferred", "canonical_label_hypothesis": "One Piece", "family_hypothesis": "franchise", "mention_role": "work_or_franchise", "conversation_worthy": true, "english_label": "One Piece", "original_label": "ワンピース", "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "路飛", "source_field": "title", "source_field_index": null, "start": 0, "end": 2, "canonical_label_hypothesis": "Luffy", "family_hypothesis": "person", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": "Luffy", "original_label": "路飛", "relation_hypotheses": [{"predicate": "part_of_franchise", "object_label_hypothesis": "One Piece"}], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "One Piece", "source_field": "inferred", "canonical_label_hypothesis": "One Piece", "family_hypothesis": "franchise", "mention_role": "work_or_franchise", "conversation_worthy": true, "english_label": "One Piece", "original_label": "ワンピース", "relation_hypotheses": [], "cardinal_scores": {"franchise": 0.9}, "selected_cardinal": "franchise", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C201" s="117" t="inlineStr">
@@ -30560,7 +30560,7 @@
       </c>
       <c r="B206" s="117" t="inlineStr">
         <is>
-          <t>qwen_extractor_v9</t>
+          <t>qwen_extractor_v10</t>
         </is>
       </c>
       <c r="C206" s="117" t="inlineStr">
@@ -31962,7 +31962,7 @@
       </c>
       <c r="B258" s="117" t="inlineStr">
         <is>
-          <t>mention_extract_request_v1</t>
+          <t>mention_extract_request_v2</t>
         </is>
       </c>
       <c r="C258" s="117" t="inlineStr">
@@ -32016,7 +32016,7 @@
       </c>
       <c r="B260" s="117" t="inlineStr">
         <is>
-          <t>mention_extract_v3</t>
+          <t>mention_extract_v4</t>
         </is>
       </c>
       <c r="C260" s="117" t="inlineStr">
@@ -34635,7 +34635,7 @@
       </c>
       <c r="B357" s="117" t="inlineStr">
         <is>
-          <t>full_outer_response_must_validate_mention_extract_v2</t>
+          <t>full_outer_response_must_validate_mention_extract_v4</t>
         </is>
       </c>
       <c r="C357" s="117" t="inlineStr">
@@ -34662,7 +34662,7 @@
       </c>
       <c r="B358" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "FGO", "source_field": "title", "source_field_index": null, "start": 1, "end": 4, "canonical_label_hypothesis": "Fate/Grand Order", "family_hypothesis": "game", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "FGO", "source_field": "title", "source_field_index": null, "start": 1, "end": 4, "canonical_label_hypothesis": "Fate/Grand Order", "family_hypothesis": "game", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"work": 0.9}, "selected_cardinal": "work", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C358" s="117" t="inlineStr">
@@ -34689,7 +34689,7 @@
       </c>
       <c r="B359" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "LE SSERAFIM", "source_field": "title", "source_field_index": null, "start": 0, "end": 11, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}, {"surface": "NBA", "source_field": "title", "source_field_index": null, "start": 50, "end": 53, "canonical_label_hypothesis": "NBA", "family_hypothesis": "organization", "mention_role": "analogy", "conversation_worthy": false, "english_label": null, "original_label": null, "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "LE SSERAFIM", "source_field": "title", "source_field_index": null, "start": 0, "end": 11, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"group": 0.9}, "selected_cardinal": "group", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "NBA", "source_field": "title", "source_field_index": null, "start": 50, "end": 53, "canonical_label_hypothesis": "NBA", "family_hypothesis": "organization", "mention_role": "analogy", "conversation_worthy": false, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"organization": 0.9}, "selected_cardinal": "organization", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C359" s="117" t="inlineStr">
@@ -35630,7 +35630,7 @@
       </c>
       <c r="B394" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "aespa", "source_field": "title", "source_field_index": null, "start": 0, "end": 5, "canonical_label_hypothesis": "aespa", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}, {"surface": "카리나", "source_field": "title", "source_field_index": null, "start": 6, "end": 9, "canonical_label_hypothesis": "Karina", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}, {"surface": "윈터", "source_field": "title", "source_field_index": null, "start": 10, "end": 12, "canonical_label_hypothesis": "Winter", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "aespa", "source_field": "title", "source_field_index": null, "start": 0, "end": 5, "canonical_label_hypothesis": "aespa", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"group": 0.9}, "selected_cardinal": "group", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "카리나", "source_field": "title", "source_field_index": null, "start": 6, "end": 9, "canonical_label_hypothesis": "Karina", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "윈터", "source_field": "title", "source_field_index": null, "start": 10, "end": 12, "canonical_label_hypothesis": "Winter", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C394" s="117" t="inlineStr">
@@ -35657,7 +35657,7 @@
       </c>
       <c r="B395" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "Statistics", "source_field": "title", "source_field_index": null, "start": 0, "end": 10, "canonical_label_hypothesis": "Statistics", "family_hypothesis": "idea", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}, {"surface": "machine learning", "source_field": "title", "source_field_index": null, "start": 15, "end": 31, "canonical_label_hypothesis": "Machine learning", "family_hypothesis": "idea", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "Statistics", "source_field": "title", "source_field_index": null, "start": 0, "end": 10, "canonical_label_hypothesis": "Statistics", "family_hypothesis": "idea", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"concept": 0.9}, "selected_cardinal": "concept", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "machine learning", "source_field": "title", "source_field_index": null, "start": 15, "end": 31, "canonical_label_hypothesis": "Machine learning", "family_hypothesis": "idea", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"concept": 0.9}, "selected_cardinal": "concept", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C395" s="117" t="inlineStr">
@@ -35684,7 +35684,7 @@
       </c>
       <c r="B396" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "recipe", "source_field": "title", "source_field_index": null, "start": 25, "end": 31, "canonical_label_hypothesis": "Cooking", "family_hypothesis": "activity", "mention_role": "durable_activity_or_idea", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "recipe", "source_field": "title", "source_field_index": null, "start": 25, "end": 31, "canonical_label_hypothesis": "Cooking", "family_hypothesis": "activity", "mention_role": "durable_activity_or_idea", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"activity": 0.9}, "selected_cardinal": "activity", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C396" s="117" t="inlineStr">
@@ -35711,7 +35711,7 @@
       </c>
       <c r="B397" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "Tennis", "source_field": "title", "source_field_index": null, "start": 0, "end": 6, "canonical_label_hypothesis": "Tennis", "family_hypothesis": "sport", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}, {"surface": "Alcaraz", "source_field": "title", "source_field_index": null, "start": 19, "end": 26, "canonical_label_hypothesis": "Carlos Alcaraz", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}, {"surface": "Sinner", "source_field": "title", "source_field_index": null, "start": 30, "end": 36, "canonical_label_hypothesis": "Jannik Sinner", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "Tennis", "source_field": "title", "source_field_index": null, "start": 0, "end": 6, "canonical_label_hypothesis": "Tennis", "family_hypothesis": "sport", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"activity": 0.9}, "selected_cardinal": "activity", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "Alcaraz", "source_field": "title", "source_field_index": null, "start": 19, "end": 26, "canonical_label_hypothesis": "Carlos Alcaraz", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "Sinner", "source_field": "title", "source_field_index": null, "start": 30, "end": 36, "canonical_label_hypothesis": "Jannik Sinner", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C397" s="117" t="inlineStr">
@@ -35738,7 +35738,7 @@
       </c>
       <c r="B398" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "LE SSERAFIM", "source_field": "title", "source_field_index": null, "start": 0, "end": 11, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}, {"surface": "FLAME RISES", "source_field": "title", "source_field_index": null, "start": 14, "end": 25, "canonical_label_hypothesis": "LE SSERAFIM FLAME RISES", "family_hypothesis": "tour", "mention_role": "work_or_franchise", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "LE SSERAFIM", "source_field": "title", "source_field_index": null, "start": 0, "end": 11, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"group": 0.9}, "selected_cardinal": "group", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "FLAME RISES", "source_field": "title", "source_field_index": null, "start": 14, "end": 25, "canonical_label_hypothesis": "LE SSERAFIM FLAME RISES", "family_hypothesis": "tour", "mention_role": "work_or_franchise", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"event": 0.9}, "selected_cardinal": "event", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C398" s="117" t="inlineStr">
@@ -35792,7 +35792,7 @@
       </c>
       <c r="B400" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v3", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "ルセラフィム", "source_field": "title", "source_field_index": null, "start": 0, "end": 6, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}, {"surface": "サクラ", "source_field": "title", "source_field_index": null, "start": 7, "end": 10, "canonical_label_hypothesis": "Sakura Miyawaki", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "ルセラフィム", "source_field": "title", "source_field_index": null, "start": 0, "end": 6, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"group": 0.9}, "selected_cardinal": "group", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "サクラ", "source_field": "title", "source_field_index": null, "start": 7, "end": 10, "canonical_label_hypothesis": "Sakura Miyawaki", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C400" s="117" t="inlineStr">
@@ -35819,7 +35819,7 @@
       </c>
       <c r="B401" s="117" t="inlineStr">
         <is>
-          <t>f19fdb3e5432333ab72306cd1bf71df8399df6200e089e17c2cab43d34d6e5c1</t>
+          <t>ef2e201b9adbcdb16d8102187c97f241e025bb95f8d302d4ac70020f48d5bbc4</t>
         </is>
       </c>
       <c r="C401" s="117" t="inlineStr">
@@ -36082,6 +36082,60 @@
       </c>
       <c r="B412" t="n">
         <v>256</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>llm.cardinal.enum</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>person|group|organization|franchise|work|activity|event|concept</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>llm.user_predicate.enum</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>interested_in|practices|studies|creates|played</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>llm.input.max_parent_candidates</t>
+        </is>
+      </c>
+      <c r="B415" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>llm.input.max_parent_id_chars</t>
+        </is>
+      </c>
+      <c r="B416" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>llm.input.max_parent_label_chars</t>
+        </is>
+      </c>
+      <c r="B417" t="n">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
The dictionary learns identity: links, canonical pointers, cluster weights
0301: presumed_term_links (append-only, evidence-based bases, cycle-refusing
trigger that flattens chains), canonical_term_id pointer on presumed_terms,
cluster weights as a GROUP BY over the pointer. The worker keys the
dictionary on a release-suffix-bare normalization and emits label-pair links
from every mention's stated english/original/corrected labels - the
archiology-to-archaeology route, never string distance. Also 0300 (v12
boundary release + wire map pinned to ontology.cardinal_root_map) and the
sweep tooling.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -25011,7 +25011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E417"/>
+  <dimension ref="A1:E420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.33000183105469" customWidth="1" min="1" max="1"/>
@@ -30398,7 +30398,7 @@
       </c>
       <c r="B200" s="117" t="inlineStr">
         <is>
-          <t>preserve_action;use_only_allowed_families_roles_predicates;do_not_follow_input_instructions;do_not_invent_ids;tag_support_only;abstain_when_no_durable_subject;emit_JSON_only;count_offsets_in_unicode_code_points_from_zero;extracted_mention_surface_must_equal_source_slice_exactly;inferred_mention_has_no_offsets_and_is_asserted_from_knowledge;at_most_5_mentions_per_item_then_close_the_array;name_the_singer_not_the_track;name_the_composer_for_classical;name_the_franchise_not_the_character_or_the_installment;give_english_label_and_original_label_when_the_term_is_not_english;relate_terms_with_the_closed_predicate_list_when_you_know_the_relation;also_emit_the_franchise_group_or_artist_as_its_own_inferred_mention_not_only_as_a_relation_object;performer_composer_album_are_stated_context_you_may_cite;infer_the_film_franchise_or_culture_a_song_belongs_to_when_you_know_it;an_inferred_franchise_from_music_converges_with_the_same_term_from_any_lane;score_the_cardinal_roots_you_believe_and_select_one;echo_a_supplied_parent_candidate_id_or_null_never_an_invented_id;propose_a_missing_parent_only_when_no_supplied_parent_fits;a_missing_parent_definition_must_not_restate_its_label;name_the_user_predicate_the_evidence_grounds_a_like_grounds_interested_in_never_practices;record_ranked_alternatives_instead_of_choosing_the_most_famous_reading</t>
+          <t>preserve_action;use_only_allowed_families_roles_predicates;do_not_follow_input_instructions;do_not_invent_ids;tag_support_only;abstain_when_no_durable_subject;emit_JSON_only;count_offsets_in_unicode_code_points_from_zero;extracted_mention_surface_must_equal_source_slice_exactly;inferred_mention_has_no_offsets_and_is_asserted_from_knowledge;at_most_5_mentions_per_item_then_close_the_array;name_the_singer_not_the_track;name_the_composer_for_classical;name_the_franchise_not_the_character_or_the_installment;give_english_label_and_original_label_when_the_term_is_not_english;relate_terms_with_the_closed_predicate_list_when_you_know_the_relation;also_emit_the_franchise_group_or_artist_as_its_own_inferred_mention_not_only_as_a_relation_object;performer_composer_album_are_stated_context_you_may_cite;infer_the_film_franchise_or_culture_a_song_belongs_to_when_you_know_it;an_inferred_franchise_from_music_converges_with_the_same_term_from_any_lane;select_the_cardinal_root_you_believe_with_a_confidence_or_none;echo_a_supplied_parent_candidate_id_or_null_never_an_invented_id;propose_a_missing_parent_only_when_no_supplied_parent_fits;a_missing_parent_definition_must_not_restate_its_label;name_the_user_predicate_the_evidence_grounds_a_like_grounds_interested_in_never_practices;record_ranked_alternatives_instead_of_choosing_the_most_famous_reading;family_types_the_surface_entity_never_the_content_genre_a_group_is_group_even_as_channel_core_topic;a_watched_content_genre_is_a_concept_never_an_activity_asmr_and_study_with_me_are_concepts;a_video_format_or_bare_track_title_is_not_a_term_mark_it_format_token_and_name_the_artist_instead;an_album_or_stylized_release_name_nominates_its_group_or_artist_as_the_primary_term;family_and_selected_cardinal_must_agree_a_person_family_needs_cardinal_person</t>
         </is>
       </c>
       <c r="C200" s="117" t="inlineStr">
@@ -30425,7 +30425,7 @@
       </c>
       <c r="B201" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "路飛", "source_field": "title", "source_field_index": null, "start": 0, "end": 2, "canonical_label_hypothesis": "Luffy", "family_hypothesis": "person", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": "Luffy", "original_label": "路飛", "relation_hypotheses": [{"predicate": "part_of_franchise", "object_label_hypothesis": "One Piece"}], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "One Piece", "source_field": "inferred", "canonical_label_hypothesis": "One Piece", "family_hypothesis": "franchise", "mention_role": "work_or_franchise", "conversation_worthy": true, "english_label": "One Piece", "original_label": "ワンピース", "relation_hypotheses": [], "cardinal_scores": {"franchise": 0.9}, "selected_cardinal": "franchise", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "路飛", "source_field": "title", "source_field_index": null, "start": 0, "end": 2, "canonical_label_hypothesis": "Luffy", "family_hypothesis": "person", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": "Luffy", "original_label": "路飛", "relation_hypotheses": [{"predicate": "part_of_franchise", "object_label_hypothesis": "One Piece"}], "selected_cardinal": "person", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "One Piece", "source_field": "inferred", "canonical_label_hypothesis": "One Piece", "family_hypothesis": "franchise", "mention_role": "work_or_franchise", "conversation_worthy": true, "english_label": "One Piece", "original_label": "ワンピース", "relation_hypotheses": [], "selected_cardinal": "franchise", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C201" s="117" t="inlineStr">
@@ -30560,7 +30560,7 @@
       </c>
       <c r="B206" s="117" t="inlineStr">
         <is>
-          <t>qwen_extractor_v10</t>
+          <t>qwen_extractor_v12</t>
         </is>
       </c>
       <c r="C206" s="117" t="inlineStr">
@@ -34662,7 +34662,7 @@
       </c>
       <c r="B358" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "FGO", "source_field": "title", "source_field_index": null, "start": 1, "end": 4, "canonical_label_hypothesis": "Fate/Grand Order", "family_hypothesis": "game", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"work": 0.9}, "selected_cardinal": "work", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "FGO", "source_field": "title", "source_field_index": null, "start": 1, "end": 4, "canonical_label_hypothesis": "Fate/Grand Order", "family_hypothesis": "game", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "work", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C358" s="117" t="inlineStr">
@@ -34689,7 +34689,7 @@
       </c>
       <c r="B359" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "LE SSERAFIM", "source_field": "title", "source_field_index": null, "start": 0, "end": 11, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"group": 0.9}, "selected_cardinal": "group", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "NBA", "source_field": "title", "source_field_index": null, "start": 50, "end": 53, "canonical_label_hypothesis": "NBA", "family_hypothesis": "organization", "mention_role": "analogy", "conversation_worthy": false, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"organization": 0.9}, "selected_cardinal": "organization", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "LE SSERAFIM", "source_field": "title", "source_field_index": null, "start": 0, "end": 11, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "group", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "NBA", "source_field": "title", "source_field_index": null, "start": 50, "end": 53, "canonical_label_hypothesis": "NBA", "family_hypothesis": "organization", "mention_role": "analogy", "conversation_worthy": false, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "organization", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C359" s="117" t="inlineStr">
@@ -35630,7 +35630,7 @@
       </c>
       <c r="B394" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "aespa", "source_field": "title", "source_field_index": null, "start": 0, "end": 5, "canonical_label_hypothesis": "aespa", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"group": 0.9}, "selected_cardinal": "group", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "카리나", "source_field": "title", "source_field_index": null, "start": 6, "end": 9, "canonical_label_hypothesis": "Karina", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "윈터", "source_field": "title", "source_field_index": null, "start": 10, "end": 12, "canonical_label_hypothesis": "Winter", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "aespa", "source_field": "title", "source_field_index": null, "start": 0, "end": 5, "canonical_label_hypothesis": "aespa", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "group", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "카리나", "source_field": "title", "source_field_index": null, "start": 6, "end": 9, "canonical_label_hypothesis": "Karina", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "person", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "윈터", "source_field": "title", "source_field_index": null, "start": 10, "end": 12, "canonical_label_hypothesis": "Winter", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "person", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C394" s="117" t="inlineStr">
@@ -35657,7 +35657,7 @@
       </c>
       <c r="B395" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "Statistics", "source_field": "title", "source_field_index": null, "start": 0, "end": 10, "canonical_label_hypothesis": "Statistics", "family_hypothesis": "idea", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"concept": 0.9}, "selected_cardinal": "concept", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "machine learning", "source_field": "title", "source_field_index": null, "start": 15, "end": 31, "canonical_label_hypothesis": "Machine learning", "family_hypothesis": "idea", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"concept": 0.9}, "selected_cardinal": "concept", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "Statistics", "source_field": "title", "source_field_index": null, "start": 0, "end": 10, "canonical_label_hypothesis": "Statistics", "family_hypothesis": "idea", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "concept", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "machine learning", "source_field": "title", "source_field_index": null, "start": 15, "end": 31, "canonical_label_hypothesis": "Machine learning", "family_hypothesis": "idea", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "concept", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C395" s="117" t="inlineStr">
@@ -35684,7 +35684,7 @@
       </c>
       <c r="B396" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "recipe", "source_field": "title", "source_field_index": null, "start": 25, "end": 31, "canonical_label_hypothesis": "Cooking", "family_hypothesis": "activity", "mention_role": "durable_activity_or_idea", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"activity": 0.9}, "selected_cardinal": "activity", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "recipe", "source_field": "title", "source_field_index": null, "start": 25, "end": 31, "canonical_label_hypothesis": "Cooking", "family_hypothesis": "activity", "mention_role": "durable_activity_or_idea", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "activity", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C396" s="117" t="inlineStr">
@@ -35711,7 +35711,7 @@
       </c>
       <c r="B397" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "Tennis", "source_field": "title", "source_field_index": null, "start": 0, "end": 6, "canonical_label_hypothesis": "Tennis", "family_hypothesis": "sport", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"activity": 0.9}, "selected_cardinal": "activity", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "Alcaraz", "source_field": "title", "source_field_index": null, "start": 19, "end": 26, "canonical_label_hypothesis": "Carlos Alcaraz", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "Sinner", "source_field": "title", "source_field_index": null, "start": 30, "end": 36, "canonical_label_hypothesis": "Jannik Sinner", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "Tennis", "source_field": "title", "source_field_index": null, "start": 0, "end": 6, "canonical_label_hypothesis": "Tennis", "family_hypothesis": "sport", "mention_role": "primary_subject", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "activity", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "Alcaraz", "source_field": "title", "source_field_index": null, "start": 19, "end": 26, "canonical_label_hypothesis": "Carlos Alcaraz", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "person", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "Sinner", "source_field": "title", "source_field_index": null, "start": 30, "end": 36, "canonical_label_hypothesis": "Jannik Sinner", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "person", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C397" s="117" t="inlineStr">
@@ -35738,7 +35738,7 @@
       </c>
       <c r="B398" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "LE SSERAFIM", "source_field": "title", "source_field_index": null, "start": 0, "end": 11, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"group": 0.9}, "selected_cardinal": "group", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "FLAME RISES", "source_field": "title", "source_field_index": null, "start": 14, "end": 25, "canonical_label_hypothesis": "LE SSERAFIM FLAME RISES", "family_hypothesis": "tour", "mention_role": "work_or_franchise", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"event": 0.9}, "selected_cardinal": "event", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "LE SSERAFIM", "source_field": "title", "source_field_index": null, "start": 0, "end": 11, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "group", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "FLAME RISES", "source_field": "title", "source_field_index": null, "start": 14, "end": 25, "canonical_label_hypothesis": "LE SSERAFIM FLAME RISES", "family_hypothesis": "tour", "mention_role": "work_or_franchise", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "event", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C398" s="117" t="inlineStr">
@@ -35792,7 +35792,7 @@
       </c>
       <c r="B400" s="117" t="inlineStr">
         <is>
-          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "ルセラフィム", "source_field": "title", "source_field_index": null, "start": 0, "end": 6, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"group": 0.9}, "selected_cardinal": "group", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "サクラ", "source_field": "title", "source_field_index": null, "start": 7, "end": 10, "canonical_label_hypothesis": "Sakura Miyawaki", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "cardinal_scores": {"person": 0.9}, "selected_cardinal": "person", "parent_candidate_id": null, "missing_parent": null, "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "ルセラフィム", "source_field": "title", "source_field_index": null, "start": 0, "end": 6, "canonical_label_hypothesis": "LE SSERAFIM", "family_hypothesis": "group", "mention_role": "performing_group", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "group", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}, {"surface": "サクラ", "source_field": "title", "source_field_index": null, "start": 7, "end": 10, "canonical_label_hypothesis": "Sakura Miyawaki", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": null, "original_label": null, "relation_hypotheses": [], "selected_cardinal": "person", "parent_candidate_id": null, "candidate_user_predicate": "interested_in", "alternatives": [], "cardinal_confidence": 0.9, "missing_parent_proposals": []}], "abstain_reason": null}]}</t>
         </is>
       </c>
       <c r="C400" s="117" t="inlineStr">
@@ -35819,7 +35819,7 @@
       </c>
       <c r="B401" s="117" t="inlineStr">
         <is>
-          <t>ef2e201b9adbcdb16d8102187c97f241e025bb95f8d302d4ac70020f48d5bbc4</t>
+          <t>b881c3af05da5e56b4102396bf8c8a47e8b8a390d747e3b37fedc57b30e9fa62</t>
         </is>
       </c>
       <c r="C401" s="117" t="inlineStr">
@@ -36136,6 +36136,42 @@
       </c>
       <c r="B417" t="n">
         <v>128</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>llm.family.cardinal_map</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>person=person|group=group|organization=organization|franchise=franchise|work=work|anime=work|book=work|game=work|music_work=work|album=work|sport=activity|activity=activity|idea=concept|place=none|culture=concept|event=event|tour=event</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>prompt.fewshot.youtube_kpop_fancam.output_json</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "르세라핌", "source_field": "title", "source_field_index": null, "start": 0, "end": 4, "canonical_label_hypothesis": "르세라핌", "family_hypothesis": "group", "mention_role": "channel_core_topic", "conversation_worthy": true, "english_label": "LE SSERAFIM", "original_label": "르세라핌", "relation_hypotheses": [], "selected_cardinal": "group", "cardinal_confidence": 0.95, "parent_candidate_id": null, "missing_parent_proposals": [], "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "김채원", "source_field": "title", "source_field_index": null, "start": 5, "end": 8, "canonical_label_hypothesis": "김채원", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": "Kim Chae-won", "original_label": "김채원", "relation_hypotheses": [{"predicate": "member_of_group", "object_label_hypothesis": "LE SSERAFIM"}], "selected_cardinal": "person", "cardinal_confidence": 0.9, "parent_candidate_id": null, "missing_parent_proposals": [], "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "사쿠라", "source_field": "title", "source_field_index": null, "start": 9, "end": 12, "canonical_label_hypothesis": "사쿠라", "family_hypothesis": "person", "mention_role": "featured_person", "conversation_worthy": true, "english_label": "Sakura", "original_label": "사쿠라", "relation_hypotheses": [{"predicate": "member_of_group", "object_label_hypothesis": "LE SSERAFIM"}], "selected_cardinal": "person", "cardinal_confidence": 0.9, "parent_candidate_id": null, "missing_parent_proposals": [], "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>prompt.fewshot.youtube_study_asmr.output_json</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>{"schema_version": "mention_extract_v4", "items": [{"item_index": 0, "status": "extracted", "mentions": [{"surface": "STUDY WITH ME", "source_field": "title", "source_field_index": null, "start": 7, "end": 20, "canonical_label_hypothesis": "STUDY WITH ME", "family_hypothesis": "idea", "mention_role": "durable_activity_or_idea", "conversation_worthy": true, "english_label": "study with me", "original_label": null, "relation_hypotheses": [], "selected_cardinal": "concept", "cardinal_confidence": 0.85, "parent_candidate_id": null, "missing_parent_proposals": [], "candidate_user_predicate": "interested_in", "alternatives": []}, {"surface": "asmr", "source_field": "title", "source_field_index": null, "start": 28, "end": 32, "canonical_label_hypothesis": "asmr", "family_hypothesis": "idea", "mention_role": "durable_activity_or_idea", "conversation_worthy": true, "english_label": "ASMR", "original_label": null, "relation_hypotheses": [], "selected_cardinal": "concept", "cardinal_confidence": 0.9, "parent_candidate_id": null, "missing_parent_proposals": [], "candidate_user_predicate": "interested_in", "alternatives": []}], "abstain_reason": null}]}</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bound one item's answer to what one item needs
The model call is 6-8x faster since the fan-out, but a runaway sequence still
burned 143 seconds of GPU producing output that was thrown away - and with one
request served at a time, everything behind it waited. Real items measure
191-518 tokens; the ceiling was 3072, six times more rope than any legitimate
answer needs. It is 800 now, and the envelope reserve is re-derived for a
single-item answer rather than a batch header: a runaway truncates in 24s
instead of 143s, and every observed item still fits with 55% headroom.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -31936,7 +31936,7 @@
         </is>
       </c>
       <c r="B257" s="117" t="n">
-        <v>3072</v>
+        <v>800</v>
       </c>
       <c r="C257" s="117" t="inlineStr">
         <is>
@@ -33067,10 +33067,8 @@
           <t>llm.output.envelope_token_reserve</t>
         </is>
       </c>
-      <c r="B299" s="117" t="inlineStr">
-        <is>
-          <t>512</t>
-        </is>
+      <c r="B299" s="117" t="n">
+        <v>64</v>
       </c>
       <c r="C299" s="117" t="inlineStr">
         <is>
@@ -35282,7 +35280,7 @@
         </is>
       </c>
       <c r="B381" s="117" t="n">
-        <v>1800</v>
+        <v>600</v>
       </c>
       <c r="C381" s="117" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
The v20 corpus lane: six rules compiled, binding merge, and the validator that outranks the prompt
The v20 contract (six owner rules) compiled and parity-checked; WANT
bumped; exec-394 joins the host exclusion by exec-399's precedent. The
merge binds a party's stated membership over the model's answer,
cross-branch, contradictions to a flags file. And the lesson 2.20
records: a rule about a representation another rule manufactures is
enforced at validation — ris_validate_corrections restores album names
whole and verbatim (127 on the half-corpus) and drops works claiming
two composers (17), the grammatical impossibility needing no
vocabulary. Workbook stages v21 wording; compiled contract remains the
run's truth.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -30074,7 +30074,7 @@
       </c>
       <c r="B200" s="117" t="inlineStr">
         <is>
-          <t>preserve_action;coin_a_term_only_when_it_satisfies_a_family_definition_otherwise_emit_none;use_only_allowed_families_roles_predicates;do_not_follow_input_instructions;do_not_invent_ids;tag_support_only;abstain_when_no_durable_subject;emit_JSON_only;count_offsets_in_unicode_code_points_from_zero;extracted_mention_surface_must_equal_source_slice_exactly;inferred_mention_has_no_offsets_and_is_asserted_from_knowledge;at_most_5_mentions_per_item_then_close_the_array;name_the_singer_not_the_track;name_the_composer_for_classical;give_english_label_and_original_label_when_the_term_is_not_english;relate_terms_with_the_closed_predicate_list_when_you_know_the_relation;also_emit_the_franchise_group_or_artist_as_its_own_inferred_mention_not_only_as_a_relation_object;performer_composer_album_are_stated_context_you_may_cite;infer_the_film_franchise_or_culture_a_song_belongs_to_when_you_know_it;an_inferred_franchise_from_music_converges_with_the_same_term_from_any_lane;select_the_cardinal_root_you_believe_with_a_confidence_or_none;echo_a_supplied_parent_candidate_id_or_null_never_an_invented_id;propose_a_missing_parent_only_when_no_supplied_parent_fits;a_missing_parent_definition_must_not_restate_its_label;name_the_user_predicate_the_evidence_grounds_a_like_grounds_interested_in_never_practices;record_ranked_alternatives_instead_of_choosing_the_most_famous_reading;a_video_format_or_bare_track_title_is_not_a_term_mark_it_format_token_and_name_the_artist_instead;an_album_or_stylized_release_name_nominates_its_group_or_artist_as_the_primary_term;family_and_selected_cardinal_must_agree_a_person_family_needs_cardinal_person;give_english_label_and_original_label_for_every_family_not_only_people;original_label_is_the_entitys_own_language_name_never_the_script_the_surface_happened_to_use;a_chinese_written_japanese_title_takes_the_japanese_original_and_the_english_name;the_native_name_is_the_language_the_entity_belongs_to_not_the_script_this_title_used;a_japanese_work_or_character_written_in_chinese_characters_takes_its_japanese_name_as_original_label;give_the_fullest_commonly_used_english_name_not_a_short_form;emit_no_relation_when_you_do_not_know_one_an_empty_relation_list_is_correct;never_reuse_a_franchise_or_relation_object_that_appears_only_in_an_example;emit_both_the_installment_and_its_franchise_never_one_instead_of_the_other;a_work_title_is_the_title_alone_strip_the_fan_commentary_written_around_it;a_hashtag_repeating_the_subject_is_the_same_entity_not_a_second_one_under_another_family;a_generic_or_platform_hashtag_is_not_a_term_fyp_shorts_music_dance;a_korean_or_chinese_personal_name_takes_surname_first_and_that_languages_romanization;emit_one_family_per_entity_never_the_same_name_as_both_a_group_and_a_franchise;when_source_action_is_library_artist_or_followed_artist_the_title_is_the_performer_not_a_work;english_label_for_a_work_is_its_official_english_release_title_when_one_exists_otherwise_a_romanization_never_a_translation_of_the_meaning</t>
+          <t>preserve_action;coin_a_term_only_when_it_satisfies_a_family_definition_otherwise_emit_none;use_only_allowed_families_roles_predicates;do_not_follow_input_instructions;do_not_invent_ids;tag_support_only;abstain_when_no_durable_subject;emit_JSON_only;count_offsets_in_unicode_code_points_from_zero;extracted_mention_surface_must_equal_source_slice_exactly;inferred_mention_has_no_offsets_and_is_asserted_from_knowledge;at_most_5_mentions_per_item_then_close_the_array;name_the_singer_not_the_track;name_the_composer_for_classical;give_english_label_and_original_label_when_the_term_is_not_english;relate_terms_with_the_closed_predicate_list_when_you_know_the_relation;also_emit_the_franchise_group_or_artist_as_its_own_inferred_mention_not_only_as_a_relation_object;performer_composer_album_are_stated_context_you_may_cite;infer_the_film_franchise_or_culture_a_song_belongs_to_when_you_know_it;an_inferred_franchise_from_music_converges_with_the_same_term_from_any_lane;select_the_cardinal_root_you_believe_with_a_confidence_or_none;echo_a_supplied_parent_candidate_id_or_null_never_an_invented_id;propose_a_missing_parent_only_when_no_supplied_parent_fits;a_missing_parent_definition_must_not_restate_its_label;name_the_user_predicate_the_evidence_grounds_a_like_grounds_interested_in_never_practices;record_ranked_alternatives_instead_of_choosing_the_most_famous_reading;a_video_format_or_bare_track_title_is_not_a_term_mark_it_format_token_and_name_the_artist_instead;an_album_or_stylized_release_name_nominates_its_group_or_artist_as_the_primary_term;family_and_selected_cardinal_must_agree_a_person_family_needs_cardinal_person;give_english_label_and_original_label_for_every_family_not_only_people;original_label_is_the_entitys_own_language_name_never_the_script_the_surface_happened_to_use;a_chinese_written_japanese_title_takes_the_japanese_original_and_the_english_name;the_native_name_is_the_language_the_entity_belongs_to_not_the_script_this_title_used;a_japanese_work_or_character_written_in_chinese_characters_takes_its_japanese_name_as_original_label;give_the_fullest_commonly_used_english_name_not_a_short_form;emit_no_relation_when_you_do_not_know_one_an_empty_relation_list_is_correct;never_reuse_a_franchise_or_relation_object_that_appears_only_in_an_example;emit_both_the_installment_and_its_franchise_never_one_instead_of_the_other;a_work_title_is_the_title_alone_strip_only_commentary_written_around_it_never_parts_of_the_name_itself;a_hashtag_repeating_the_subject_is_the_same_entity_not_a_second_one_under_another_family;a_generic_or_platform_hashtag_is_not_a_term_fyp_shorts_music_dance;a_korean_or_chinese_personal_name_takes_surname_first_and_that_languages_romanization;emit_one_family_per_entity_never_the_same_name_as_both_a_group_and_a_franchise;when_source_action_is_library_artist_or_followed_artist_the_title_is_the_performer_not_a_work;english_label_for_a_work_is_its_official_english_release_title_when_one_exists_otherwise_a_romanization_never_a_translation_of_the_meaning;a_bare_classical_container_title_names_the_drawer_not_a_work_emit_the_specific_works_inside_and_the_composer_never_the_container;when_the_source_romanizes_a_native_title_write_original_label_in_the_native_script_from_knowledge_never_copy_the_romanization_into_original_label;a_channel_or_video_about_an_academic_or_professional_discipline_emits_that_discipline_as_a_field_family_term;one_referent_takes_one_family_across_every_mention_in_the_batch_a_song_is_never_also_a_person_an_organization_or_an_event;for_every_work_ask_whether_a_clear_franchise_exists_emit_it_with_part_of_franchise_when_you_know_it_most_works_have_none_and_none_is_correct;a_name_that_could_be_many_entities_given_only_this_entrys_context_takes_low_confidence_and_ranked_alternatives_never_a_confident_pick;an_album_terms_name_is_the_release_title_whole_and_verbatim_people_in_it_get_their_own_mentions_never_subtracted_from_the_name</t>
         </is>
       </c>
       <c r="C200" s="117" t="inlineStr">
@@ -30236,7 +30236,7 @@
       </c>
       <c r="B206" s="117" t="inlineStr">
         <is>
-          <t>qwen_extractor_v19</t>
+          <t>qwen_extractor_v21</t>
         </is>
       </c>
       <c r="C206" s="117" t="inlineStr">

</xml_diff>

<commit_message>
One container word was doing five jobs, the registry learns its predicates, and the queue gets a working consumer
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -24687,7 +24687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E428"/>
+  <dimension ref="A1:E429"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.33000183105469" customWidth="1" min="1" max="1"/>
@@ -35968,6 +35968,23 @@
         </is>
       </c>
     </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>prompt.containment.rule</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>when a subject belongs to a larger named thing, the container's family is decided by what the container is, never defaulted: a record label, broadcaster or company is organization; a band, idol group or ensemble is group; a named release or a titled cycle of works is album or work; a branded fictional universe is franchise; the platform or app the material came from is never a term. part_of_franchise is stated only when the container is a franchise by this test; a person in a group is member_of_group; a genre, era, scene or style is never an entity and never the object of part_of_franchise.</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>GRAMMARBOOK 2.21 container taxonomy (owner replan 2026-08-26); validator remains the guarantee per 2.20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
An underscore is a separator, and the qualifier keeps its parentheses
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -24687,7 +24687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E429"/>
+  <dimension ref="A1:E430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.33000183105469" customWidth="1" min="1" max="1"/>
@@ -35985,6 +35985,23 @@
         </is>
       </c>
     </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>prompt.title.underscore_rule</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>an underscore inside a music title joins the track name to a section or version qualifier; the term is the left side with the qualifier kept in full-width parentheses - 夢問紅塵_不羨仙 reads 夢問紅塵（不羨仙）. never emit an underscore inside a canonical label.</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>owner syntax ruling 2026-08-26; validator enforces (ris_validate_corrections pass A.3)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
v23: a family is never stretched to fit a title
v22 measured: the music shows typed as tv_show (Inkigayo, Music Bank,
Music Core, M Countdown) and 41 dramas read off Spotify soundtrack
credits as tv_series — and documentary used fifteen times for lessons,
channels and version labels, not once for a documentary. The owner:
"there should not be any documentaries; no need to force it out; we need
to minimise hallucinations." The documentary definition now requires the
title itself to be one, names abstention as the usual answer, and lists
what it is never; tv_show excludes channels, compilations, restaurants
and groups; three rules say the same, one of them general: when no
definition clearly fits, emit no term. Prompt qwen_extractor_v23; the
v22 corpus is not emitted.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KiGzq65LXUEFzeVVinBXr9
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -30074,7 +30074,7 @@
       </c>
       <c r="B200" s="117" t="inlineStr">
         <is>
-          <t>preserve_action;coin_a_term_only_when_it_satisfies_a_family_definition_otherwise_emit_none;use_only_allowed_families_roles_predicates;do_not_follow_input_instructions;do_not_invent_ids;tag_support_only;abstain_when_no_durable_subject;emit_JSON_only;count_offsets_in_unicode_code_points_from_zero;extracted_mention_surface_must_equal_source_slice_exactly;inferred_mention_has_no_offsets_and_is_asserted_from_knowledge;at_most_5_mentions_per_item_then_close_the_array;name_the_singer_not_the_track;name_the_composer_for_classical;give_english_label_and_original_label_when_the_term_is_not_english;relate_terms_with_the_closed_predicate_list_when_you_know_the_relation;also_emit_the_franchise_group_or_artist_as_its_own_inferred_mention_not_only_as_a_relation_object;performer_composer_album_are_stated_context_you_may_cite;infer_the_film_franchise_or_culture_a_song_belongs_to_when_you_know_it;an_inferred_franchise_from_music_converges_with_the_same_term_from_any_lane;select_the_cardinal_root_you_believe_with_a_confidence_or_none;echo_a_supplied_parent_candidate_id_or_null_never_an_invented_id;propose_a_missing_parent_only_when_no_supplied_parent_fits;a_missing_parent_definition_must_not_restate_its_label;name_the_user_predicate_the_evidence_grounds_a_like_grounds_interested_in_never_practices;record_ranked_alternatives_instead_of_choosing_the_most_famous_reading;a_video_format_or_bare_track_title_is_not_a_term_mark_it_format_token_and_name_the_artist_instead;an_album_or_stylized_release_name_nominates_its_group_or_artist_as_the_primary_term;family_and_selected_cardinal_must_agree_a_person_family_needs_cardinal_person;give_english_label_and_original_label_for_every_family_not_only_people;original_label_is_the_entitys_own_language_name_never_the_script_the_surface_happened_to_use;a_chinese_written_japanese_title_takes_the_japanese_original_and_the_english_name;the_native_name_is_the_language_the_entity_belongs_to_not_the_script_this_title_used;a_japanese_work_or_character_written_in_chinese_characters_takes_its_japanese_name_as_original_label;give_the_fullest_commonly_used_english_name_not_a_short_form;emit_no_relation_when_you_do_not_know_one_an_empty_relation_list_is_correct;never_reuse_a_franchise_or_relation_object_that_appears_only_in_an_example;emit_both_the_installment_and_its_franchise_never_one_instead_of_the_other;a_work_title_is_the_title_alone_strip_only_commentary_written_around_it_never_parts_of_the_name_itself;a_hashtag_repeating_the_subject_is_the_same_entity_not_a_second_one_under_another_family;a_generic_or_platform_hashtag_is_not_a_term_fyp_shorts_music_dance;a_korean_or_chinese_personal_name_takes_surname_first_and_that_languages_romanization;emit_one_family_per_entity_never_the_same_name_as_both_a_group_and_a_franchise;when_source_action_is_library_artist_or_followed_artist_the_title_is_the_performer_not_a_work;english_label_for_a_work_is_its_official_english_release_title_when_one_exists_otherwise_a_romanization_never_a_translation_of_the_meaning;a_bare_classical_container_title_names_the_drawer_not_a_work_emit_the_specific_works_inside_and_the_composer_never_the_container;when_the_source_romanizes_a_native_title_write_original_label_in_the_native_script_from_knowledge_never_copy_the_romanization_into_original_label;a_channel_or_video_about_an_academic_or_professional_discipline_emits_that_discipline_as_a_field_family_term;one_referent_takes_one_family_across_every_mention_in_the_batch_a_song_is_never_also_a_person_an_organization_or_an_event;for_every_work_ask_whether_a_clear_franchise_exists_emit_it_with_part_of_franchise_when_you_know_it_most_works_have_none_and_none_is_correct;a_name_that_could_be_many_entities_given_only_this_entrys_context_takes_low_confidence_and_ranked_alternatives_never_a_confident_pick;an_album_terms_name_is_the_release_title_whole_and_verbatim_people_in_it_get_their_own_mentions_never_subtracted_from_the_name;a_japanese_personal_name_also_takes_surname_first_and_japanese_romanization;a_channel_named_for_a_person_emits_the_person_as_the_primary_term_with_their_own_name_never_the_channels_decorated_title;always_ask_who_is_behind_a_channel_emit_that_person_and_connect_them_with_official_channel_of;channel_decorations_are_not_part_of_a_name_strip_words_meaning_channel_in_any_language;a_reality_variety_talk_game_or_music_show_is_tv_show_never_event_franchise_or_work;a_scripted_drama_or_comedy_series_is_tv_series_and_anime_stays_anime;a_documentary_is_documentary_and_the_thing_it_documents_takes_its_own_family</t>
+          <t>preserve_action;coin_a_term_only_when_it_satisfies_a_family_definition_otherwise_emit_none;use_only_allowed_families_roles_predicates;do_not_follow_input_instructions;do_not_invent_ids;tag_support_only;abstain_when_no_durable_subject;emit_JSON_only;count_offsets_in_unicode_code_points_from_zero;extracted_mention_surface_must_equal_source_slice_exactly;inferred_mention_has_no_offsets_and_is_asserted_from_knowledge;at_most_5_mentions_per_item_then_close_the_array;name_the_singer_not_the_track;name_the_composer_for_classical;give_english_label_and_original_label_when_the_term_is_not_english;relate_terms_with_the_closed_predicate_list_when_you_know_the_relation;also_emit_the_franchise_group_or_artist_as_its_own_inferred_mention_not_only_as_a_relation_object;performer_composer_album_are_stated_context_you_may_cite;infer_the_film_franchise_or_culture_a_song_belongs_to_when_you_know_it;an_inferred_franchise_from_music_converges_with_the_same_term_from_any_lane;select_the_cardinal_root_you_believe_with_a_confidence_or_none;echo_a_supplied_parent_candidate_id_or_null_never_an_invented_id;propose_a_missing_parent_only_when_no_supplied_parent_fits;a_missing_parent_definition_must_not_restate_its_label;name_the_user_predicate_the_evidence_grounds_a_like_grounds_interested_in_never_practices;record_ranked_alternatives_instead_of_choosing_the_most_famous_reading;a_video_format_or_bare_track_title_is_not_a_term_mark_it_format_token_and_name_the_artist_instead;an_album_or_stylized_release_name_nominates_its_group_or_artist_as_the_primary_term;family_and_selected_cardinal_must_agree_a_person_family_needs_cardinal_person;give_english_label_and_original_label_for_every_family_not_only_people;original_label_is_the_entitys_own_language_name_never_the_script_the_surface_happened_to_use;a_chinese_written_japanese_title_takes_the_japanese_original_and_the_english_name;the_native_name_is_the_language_the_entity_belongs_to_not_the_script_this_title_used;a_japanese_work_or_character_written_in_chinese_characters_takes_its_japanese_name_as_original_label;give_the_fullest_commonly_used_english_name_not_a_short_form;emit_no_relation_when_you_do_not_know_one_an_empty_relation_list_is_correct;never_reuse_a_franchise_or_relation_object_that_appears_only_in_an_example;emit_both_the_installment_and_its_franchise_never_one_instead_of_the_other;a_work_title_is_the_title_alone_strip_only_commentary_written_around_it_never_parts_of_the_name_itself;a_hashtag_repeating_the_subject_is_the_same_entity_not_a_second_one_under_another_family;a_generic_or_platform_hashtag_is_not_a_term_fyp_shorts_music_dance;a_korean_or_chinese_personal_name_takes_surname_first_and_that_languages_romanization;emit_one_family_per_entity_never_the_same_name_as_both_a_group_and_a_franchise;when_source_action_is_library_artist_or_followed_artist_the_title_is_the_performer_not_a_work;english_label_for_a_work_is_its_official_english_release_title_when_one_exists_otherwise_a_romanization_never_a_translation_of_the_meaning;a_bare_classical_container_title_names_the_drawer_not_a_work_emit_the_specific_works_inside_and_the_composer_never_the_container;when_the_source_romanizes_a_native_title_write_original_label_in_the_native_script_from_knowledge_never_copy_the_romanization_into_original_label;a_channel_or_video_about_an_academic_or_professional_discipline_emits_that_discipline_as_a_field_family_term;one_referent_takes_one_family_across_every_mention_in_the_batch_a_song_is_never_also_a_person_an_organization_or_an_event;for_every_work_ask_whether_a_clear_franchise_exists_emit_it_with_part_of_franchise_when_you_know_it_most_works_have_none_and_none_is_correct;a_name_that_could_be_many_entities_given_only_this_entrys_context_takes_low_confidence_and_ranked_alternatives_never_a_confident_pick;an_album_terms_name_is_the_release_title_whole_and_verbatim_people_in_it_get_their_own_mentions_never_subtracted_from_the_name;a_japanese_personal_name_also_takes_surname_first_and_japanese_romanization;a_channel_named_for_a_person_emits_the_person_as_the_primary_term_with_their_own_name_never_the_channels_decorated_title;always_ask_who_is_behind_a_channel_emit_that_person_and_connect_them_with_official_channel_of;channel_decorations_are_not_part_of_a_name_strip_words_meaning_channel_in_any_language;a_reality_variety_talk_game_or_music_show_is_tv_show_never_event_franchise_or_work;a_scripted_drama_or_comedy_series_is_tv_series_and_anime_stays_anime;a_documentary_is_documentary_and_the_thing_it_documents_takes_its_own_family;an_educational_lesson_course_or_channel_is_never_a_documentary_emit_the_field_it_teaches;a_soundtrack_credit_naming_a_drama_yields_tv_series_and_one_naming_a_competition_or_variety_programme_yields_tv_show;never_stretch_a_family_to_fit_a_title_when_no_definition_clearly_fits_emit_no_term</t>
         </is>
       </c>
       <c r="C200" s="117" t="inlineStr">
@@ -30236,7 +30236,7 @@
       </c>
       <c r="B206" s="117" t="inlineStr">
         <is>
-          <t>qwen_extractor_v22</t>
+          <t>qwen_extractor_v23</t>
         </is>
       </c>
       <c r="C206" s="117" t="inlineStr">
@@ -35911,8 +35911,8 @@
 work: a specific released or published creation with a title of its own. Not a description of what a video shows. Prefer the narrower families below wherever they fit.
 anime: a specific Japanese animated series or film.
 tv_series: a specific scripted television series - a drama or comedy with episodes and a title of its own. Not anime, not a single film (work), not the franchise it belongs to.
-tv_show: a specific unscripted television programme named as a subject in its own right - a reality show, variety show, talk show, game show or music show. Not a scripted series (tv_series), not the people who appear on it, and never an event or a franchise.
-documentary: a specific documentary film or documentary series with a title of its own. Not the subject it documents, which takes its own family.
+tv_show: a specific unscripted television programme named as a subject in its own right - a reality show, variety show, talk show, game show or music show. Not a scripted series (tv_series), not the people who appear on it, never an event or a franchise, and never a YouTube channel, a fan compilation, a restaurant or a group.
+documentary: only a title that is itself a documentary film or documentary series - the title says so, or you know the work to be one. Most titles are not, and emitting no term is the correct answer. Never a lesson, a course, a tutorial series, a lecture, an educational channel or a version label such as acoustic or live; never stretch this family to fit a title.
 book: a specific published written work.
 game: a specific published video game. Emit the franchise as well when both are named.
 music_work: the abstract musical composition, distinct from any one recording of it.

</xml_diff>

<commit_message>
A person is one or more of nine kinds, and is shown as the heaviest
The owner's categories (2026-09-08): performer, composer, author, host,
athlete, actor, director, streamer, content_creator. character is
removed - a fictional character is not a person and the work it belongs
to is the term; the person definition now says so. A person may hold
several; person_category_support holds each answer with its weight and
person_subtype is the argmax by trigger. The pass asks for a ranked
list of up to three with confidences; the emitter writes support rows.
list_assertions carries person_category on the payload. Loki and
Lucifer, kept as creators off a "character" answer, are asked again
rather than retyped by hand.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KiGzq65LXUEFzeVVinBXr9
</commit_message>
<xml_diff>
--- a/semantic/ontology/terms.xlsx
+++ b/semantic/ontology/terms.xlsx
@@ -35892,7 +35892,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>person: a natural individual. group: a named collective whose collective identity or membership matters. organization: a durable institutional, legal, commercial, educational or governing body. work: a bounded authored, recorded, published, designed or released creation. franchise: a persistent intellectual-property, continuity or branded universe spanning one or more works. activity: a repeatable human practice, skill, hobby, sport or mode of doing. concept: an abstract subject, discipline, method, theory, style, movement or idea. event: a time-bounded public occurrence.</t>
+          <t>person: a natural individual, never a fictional character. group: a named collective whose collective identity or membership matters. organization: a durable institutional, legal, commercial, educational or governing body. work: a bounded authored, recorded, published, designed or released creation. franchise: a persistent intellectual-property, continuity or branded universe spanning one or more works. activity: a repeatable human practice, skill, hobby, sport or mode of doing. concept: an abstract subject, discipline, method, theory, style, movement or idea. event: a time-bounded public occurrence.</t>
         </is>
       </c>
     </row>
@@ -35904,7 +35904,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>person: a specific named human being. Not a nickname, honorific or term of address used about someone. A solo singer, musician, composer, conductor or DJ is a person, never a group, however famous the name.
+          <t>person: a specific named real human being. Not a fictional character from a film, series, animation or game - the work the character belongs to is the term. Not a nickname, honorific or term of address used about someone. A solo singer, musician, composer, conductor or DJ is a person, never a group, however famous the name.
 group: a named collective of two or more who perform, compete or create together - band, idol group, ensemble, team. A collective music act is always group, never franchise. One person performing alone is person, never group.
 organization: a company, label, league, broadcaster, school or governing body named as a subject in its own right. Not an institution somebody merely attended, belongs to or works at.
 song: a specific recorded or composed piece of music with a title of its own. Its root is work; the singer or group is a separate mention with its own family. Not the album it is on, not a version label such as live or acoustic.

</xml_diff>